<commit_message>
Restore Excel dropdown validations (stripped by openpyxl on prev save)
Re-adds data validation for all 4 input cells:
  C9  — Country (7 options incl. Vietnam)
  C10 — Industry (7 options)
  C12 — Annual Revenue (5 bands)
  C14 — Prior Incident (Yes / No / I'm Not Sure)

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veeam-VDC-ROI-Calculator.xlsx
+++ b/Veeam-VDC-ROI-Calculator.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29080" windowHeight="16820" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ROI Calculator" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Ref" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Recovery Workflow" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROI Calculator" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ref" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Workflow" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -2462,9 +2462,9 @@
     <row r="56" ht="15" customHeight="1" s="114"/>
   </sheetData>
   <mergeCells count="44">
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="D13:F13"/>
     <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="B7:F7"/>
     <mergeCell ref="E24:F24"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="B31:F31"/>
@@ -2507,8 +2507,17 @@
     <mergeCell ref="B41:F41"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="C14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid Entry" error="Please select Yes, No, or I'm Not Sure" type="list">
+  <dataValidations count="4">
+    <dataValidation sqref="C9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid entry" error="Please select a country from the list." type="list">
+      <formula1>"Singapore,Indonesia,Thailand,Philippines,Malaysia,South Korea,Vietnam"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid entry" error="Please select an industry from the list." type="list">
+      <formula1>"Financial,Healthcare,Legal,Tech,Retail,Manufacturing,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C12" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid entry" error="Please select a revenue band from the list." type="list">
+      <formula1>"Under USD 50M,USD 50M – 500M,USD 500M – 2B,USD 2B – 10B,Over USD 10B"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid entry" error="Please select Yes, No, or I'm Not Sure." type="list">
       <formula1>"Yes,No,I'm Not Sure"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fix Excel summary sentence — separate gross ratio from net savings
Old sentence conflated 16.3× (gross risk/cost ratio) with $28.8M
(net savings), which a CFO would immediately flag as inconsistent.

New format clearly shows all four numbers:
  Annual risk exposure · Veeam cost · Protection ratio · Net savings

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Veeam-VDC-ROI-Calculator.xlsx
+++ b/Veeam-VDC-ROI-Calculator.xlsx
@@ -2424,7 +2424,7 @@
     <row r="42" ht="72" customHeight="1" s="114">
       <c r="A42" s="130" t="n"/>
       <c r="B42" s="121">
-        <f>"For every $1 invested in Veeam Data Cloud for M365, "&amp;TEXT(D37,"0.0")&amp;"× of that value is protected as expected loss avoidance — estimated "&amp;TEXT(D38,"$#,##0")&amp;" annually."&amp;IF(D37&lt;1," ⚠  Protection ratio below 1.0× at this org size — consider requesting a volume-adjusted Veeam quote.","")</f>
+        <f>"Annual risk exposure: "&amp;TEXT(D30,"$#,##0")&amp;"  ·  Veeam annual cost: "&amp;TEXT(D35,"$#,##0")&amp;"  ·  Protection ratio: "&amp;TEXT(D37,"0.0")&amp;"×  (every $1 invested covers $"&amp;TEXT(D37,"0.0")&amp;" of risk exposure)  ·  Net expected annual savings: "&amp;TEXT(D38,"$#,##0")&amp;IF(D37&lt;1," ⚠  Protection ratio below 1.0× at this org size — consider requesting a volume-adjusted Veeam quote.",".")</f>
         <v/>
       </c>
       <c r="G42" s="130" t="n"/>
@@ -2462,9 +2462,9 @@
     <row r="56" ht="15" customHeight="1" s="114"/>
   </sheetData>
   <mergeCells count="44">
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D13:F13"/>
     <mergeCell ref="B7:F7"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="D11:F11"/>
     <mergeCell ref="E24:F24"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="B31:F31"/>

</xml_diff>